<commit_message>
fix(q1): unify gravity at 9.806 and regenerate verified results
</commit_message>
<xml_diff>
--- a/results/q1_exact_dp/Q1_结果提交.xlsx
+++ b/results/q1_exact_dp/Q1_结果提交.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Q3_中继架次" sheetId="4" r:id="rId4"/>
     <sheet name="Q3_通信保障" sheetId="5" r:id="rId5"/>
     <sheet name="Q4_分区配置" sheetId="6" r:id="rId6"/>
+    <sheet name="Q1_方案对比" sheetId="7" r:id="rId10"/>
+    <sheet name="Q1_模型说明" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="151">
   <si>
     <r>
       <rPr>
@@ -664,6 +666,150 @@
   </si>
   <si>
     <t>S015-MED-01;S015-FOD-01;S015-WAT-01</t>
+  </si>
+  <si>
+    <t>objective</t>
+  </si>
+  <si>
+    <t>N-E-T</t>
+  </si>
+  <si>
+    <t>N-T-E</t>
+  </si>
+  <si>
+    <t>E-N-T</t>
+  </si>
+  <si>
+    <t>E-T-N</t>
+  </si>
+  <si>
+    <t>T-N-E</t>
+  </si>
+  <si>
+    <t>T-E-N</t>
+  </si>
+  <si>
+    <t>weighted_joint_N60_E25_T15</t>
+  </si>
+  <si>
+    <t>weighted_joint_balanced</t>
+  </si>
+  <si>
+    <t>weighted_joint_N15_E60_T25</t>
+  </si>
+  <si>
+    <t>weighted_joint_N15_E25_T60</t>
+  </si>
+  <si>
+    <t>weighted_joint_N45_E30_T25</t>
+  </si>
+  <si>
+    <t>weighted_joint_energy_dominant_N01_E98_T01</t>
+  </si>
+  <si>
+    <t>greedy_baseline</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>lexicographic</t>
+  </si>
+  <si>
+    <t>joint_weighted</t>
+  </si>
+  <si>
+    <t>greedy</t>
+  </si>
+  <si>
+    <t>sortie_weight</t>
+  </si>
+  <si>
+    <t>energy_weight</t>
+  </si>
+  <si>
+    <t>time_weight</t>
+  </si>
+  <si>
+    <t>scale_sorties</t>
+  </si>
+  <si>
+    <t>scale_energy_kWh</t>
+  </si>
+  <si>
+    <t>scale_time_h</t>
+  </si>
+  <si>
+    <t>total_sorties</t>
+  </si>
+  <si>
+    <t>total_energy_kWh</t>
+  </si>
+  <si>
+    <t>total_operation_time_h</t>
+  </si>
+  <si>
+    <t>normalized_objective</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>single-objective priority order</t>
+  </si>
+  <si>
+    <t>all three criteria included</t>
+  </si>
+  <si>
+    <t>baseline only</t>
+  </si>
+  <si>
+    <t>项目</t>
+  </si>
+  <si>
+    <t>重力加速度</t>
+  </si>
+  <si>
+    <t>算法</t>
+  </si>
+  <si>
+    <t>主方案</t>
+  </si>
+  <si>
+    <t>三目标加权</t>
+  </si>
+  <si>
+    <t>主方案结果</t>
+  </si>
+  <si>
+    <t>时间口径</t>
+  </si>
+  <si>
+    <t>最优性范围</t>
+  </si>
+  <si>
+    <t>说明</t>
+  </si>
+  <si>
+    <t>g=9.806 m/s^2，与问题二三统一</t>
+  </si>
+  <si>
+    <t>可行模式枚举 + 精确计数状态动态规划；intlinprog交叉验证</t>
+  </si>
+  <si>
+    <t>词典序：架次数 → 能耗 → 累计作业时间</t>
+  </si>
+  <si>
+    <t>J=wN*N/N0+wE*E/E0+wT*T/T0，权重和为1</t>
+  </si>
+  <si>
+    <t>18架次，59.130253926649 kWh，9.104448819143 h</t>
+  </si>
+  <si>
+    <t>模板往返时间列沿用完整架次作业时间；CSV另保留flight_time_s纯飞行时间</t>
+  </si>
+  <si>
+    <t>固定物理解释、枚举模式及数值容差下的所选目标；不代表所有偏好唯一最优</t>
   </si>
 </sst>
 </file>
@@ -1868,10 +2014,10 @@
         <v>1692.1690773290522</v>
       </c>
       <c r="H2" s="7">
-        <v>2.9175823075810157</v>
+        <v>2.9175399733426497</v>
       </c>
       <c r="I2" s="7">
-        <v>63.5302211552373</v>
+        <v>63.530750333216879</v>
       </c>
     </row>
     <row r="3">
@@ -1897,10 +2043,10 @@
         <v>1494.1690773290522</v>
       </c>
       <c r="H3" s="7">
-        <v>2.9957692627220123</v>
+        <v>2.9957264798521339</v>
       </c>
       <c r="I3" s="7">
-        <v>62.552884215974849</v>
+        <v>62.553419001848319</v>
       </c>
     </row>
     <row r="4">
@@ -1926,10 +2072,10 @@
         <v>1816.6943000984102</v>
       </c>
       <c r="H4" s="6">
-        <v>2.7134222874377589</v>
+        <v>2.7133881402010411</v>
       </c>
       <c r="I4" s="6">
-        <v>32.164442814056024</v>
+        <v>32.165296494973973</v>
       </c>
     </row>
     <row r="5">
@@ -1955,10 +2101,10 @@
         <v>2041.812384815207</v>
       </c>
       <c r="H5" s="6">
-        <v>5.7212246708574126</v>
+        <v>5.7211798054824712</v>
       </c>
       <c r="I5" s="6">
-        <v>28.484691614282344</v>
+        <v>28.48525243146911</v>
       </c>
     </row>
     <row r="6">
@@ -1984,10 +2130,10 @@
         <v>2080.5233035436581</v>
       </c>
       <c r="H6" s="6">
-        <v>2.7799174679726693</v>
+        <v>2.7798347763964069</v>
       </c>
       <c r="I6" s="6">
-        <v>30.502063300683268</v>
+        <v>30.504130590089829</v>
       </c>
     </row>
     <row r="7">
@@ -2013,10 +2159,10 @@
         <v>2370.0913496048561</v>
       </c>
       <c r="H7" s="6">
-        <v>5.7649651151972972</v>
+        <v>5.7648566851506047</v>
       </c>
       <c r="I7" s="6">
-        <v>27.937936060033785</v>
+        <v>27.939291435617442</v>
       </c>
     </row>
     <row r="8">
@@ -2042,10 +2188,10 @@
         <v>2301.0566924831601</v>
       </c>
       <c r="H8" s="6">
-        <v>6.1529320189069754</v>
+        <v>6.1528598719220176</v>
       </c>
       <c r="I8" s="6">
-        <v>23.088349763662809</v>
+        <v>23.08925160097478</v>
       </c>
     </row>
     <row r="9">
@@ -2071,10 +2217,10 @@
         <v>1877.1905245257485</v>
       </c>
       <c r="H9" s="6">
-        <v>4.2221928595068432</v>
+        <v>4.2221391566447011</v>
       </c>
       <c r="I9" s="6">
-        <v>47.222589256164461</v>
+        <v>47.223260541941237</v>
       </c>
     </row>
     <row r="10">
@@ -2100,10 +2246,10 @@
         <v>1561.553867961642</v>
       </c>
       <c r="H10" s="6">
-        <v>2.5979878649120525</v>
+        <v>2.5979349093557809</v>
       </c>
       <c r="I10" s="6">
-        <v>67.525151688599337</v>
+        <v>67.525813633052749</v>
       </c>
     </row>
     <row r="11">
@@ -2129,10 +2275,10 @@
         <v>1907.5664573299073</v>
       </c>
       <c r="H11" s="6">
-        <v>3.4108943800033673</v>
+        <v>3.4108086087645568</v>
       </c>
       <c r="I11" s="6">
-        <v>57.363820249957911</v>
+        <v>57.364892390443046</v>
       </c>
     </row>
     <row r="12">
@@ -2158,10 +2304,10 @@
         <v>2199.7012130854737</v>
       </c>
       <c r="H12" s="6">
-        <v>5.8360117114838781</v>
+        <v>5.8359572284520809</v>
       </c>
       <c r="I12" s="6">
-        <v>27.049853606451524</v>
+        <v>27.050534644348989</v>
       </c>
     </row>
     <row r="13">
@@ -2187,10 +2333,10 @@
         <v>1558.4417330887577</v>
       </c>
       <c r="H13" s="6">
-        <v>2.096233734426161</v>
+        <v>2.0962044018931136</v>
       </c>
       <c r="I13" s="6">
-        <v>47.594156639345975</v>
+        <v>47.594889952672162</v>
       </c>
     </row>
     <row r="14">
@@ -2216,10 +2362,10 @@
         <v>1555.3795658312195</v>
       </c>
       <c r="H14" s="6">
-        <v>1.8231956980899264</v>
+        <v>1.8231444995358754</v>
       </c>
       <c r="I14" s="6">
-        <v>54.42010754775184</v>
+        <v>54.421387511603115</v>
       </c>
     </row>
     <row r="15">
@@ -2245,10 +2391,10 @@
         <v>1188.4204722350105</v>
       </c>
       <c r="H15" s="6">
-        <v>1.0739517654350652</v>
+        <v>1.0739201272065426</v>
       </c>
       <c r="I15" s="6">
-        <v>73.151205864123369</v>
+        <v>73.151996819836441</v>
       </c>
     </row>
     <row r="16">
@@ -2274,10 +2420,10 @@
         <v>1922.7403507441504</v>
       </c>
       <c r="H16" s="6">
-        <v>2.7524142988016456</v>
+        <v>2.752361240693304</v>
       </c>
       <c r="I16" s="6">
-        <v>31.18964252995886</v>
+        <v>31.1909689826674</v>
       </c>
     </row>
     <row r="17">
@@ -2303,10 +2449,10 @@
         <v>1510.4723251019025</v>
       </c>
       <c r="H17" s="6">
-        <v>1.8247592723274209</v>
+        <v>1.8247168036813126</v>
       </c>
       <c r="I17" s="6">
-        <v>54.381018191814476</v>
+        <v>54.382079907967181</v>
       </c>
     </row>
     <row r="18">
@@ -2332,10 +2478,10 @@
         <v>1869.7564163814459</v>
       </c>
       <c r="H18" s="6">
-        <v>2.1403884821071424</v>
+        <v>2.1402998341980486</v>
       </c>
       <c r="I18" s="6">
-        <v>46.490287947321441</v>
+        <v>46.492504145048784</v>
       </c>
     </row>
     <row r="19">
@@ -2361,10 +2507,10 @@
         <v>1828.2766374270207</v>
       </c>
       <c r="H19" s="6">
-        <v>2.3074528242842076</v>
+        <v>2.3073813838759016</v>
       </c>
       <c r="I19" s="6">
-        <v>42.313679392894812</v>
+        <v>42.315465403102458</v>
       </c>
     </row>
   </sheetData>
@@ -6080,4 +6226,581 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="41.82421875" customWidth="true"/>
+    <col min="2" max="2" width="13.22265625" customWidth="true"/>
+    <col min="3" max="3" width="12.625" customWidth="true"/>
+    <col min="4" max="4" width="13.5234375" customWidth="true"/>
+    <col min="5" max="5" width="12.625" customWidth="true"/>
+    <col min="6" max="6" width="11.921875" customWidth="true"/>
+    <col min="7" max="7" width="17.22265625" customWidth="true"/>
+    <col min="8" max="8" width="12.125" customWidth="true"/>
+    <col min="9" max="9" width="10.82421875" customWidth="true"/>
+    <col min="10" max="10" width="16.125" customWidth="true"/>
+    <col min="11" max="11" width="19.921875" customWidth="true"/>
+    <col min="12" max="12" width="18.921875" customWidth="true"/>
+    <col min="13" max="13" width="25.22265625" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+      <c r="I2" s="0">
+        <v>18</v>
+      </c>
+      <c r="J2" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K2" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L2" s="0"/>
+      <c r="M2" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0">
+        <v>18</v>
+      </c>
+      <c r="J3" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K3" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L3" s="0"/>
+      <c r="M3" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0">
+        <v>19</v>
+      </c>
+      <c r="J4" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="K4" s="0">
+        <v>9.5666603908752492</v>
+      </c>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="0"/>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+      <c r="I5" s="0">
+        <v>19</v>
+      </c>
+      <c r="J5" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="K5" s="0">
+        <v>9.5666603908752492</v>
+      </c>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+      <c r="I6" s="0">
+        <v>18</v>
+      </c>
+      <c r="J6" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K6" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L6" s="0"/>
+      <c r="M6" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="0"/>
+      <c r="D7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0">
+        <v>18</v>
+      </c>
+      <c r="J7" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K7" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="0">
+        <v>0.14999999999999999</v>
+      </c>
+      <c r="F8" s="0">
+        <v>18</v>
+      </c>
+      <c r="G8" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H8" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I8" s="0">
+        <v>18</v>
+      </c>
+      <c r="J8" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K8" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L8" s="0">
+        <v>1.0004124233539311</v>
+      </c>
+      <c r="M8" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="0">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D9" s="0">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E9" s="0">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F9" s="0">
+        <v>18</v>
+      </c>
+      <c r="G9" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H9" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I9" s="0">
+        <v>18</v>
+      </c>
+      <c r="J9" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K9" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L9" s="0">
+        <v>1.0005498978052414</v>
+      </c>
+      <c r="M9" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="0">
+        <v>0.14999999999999999</v>
+      </c>
+      <c r="D10" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="E10" s="0">
+        <v>0.25</v>
+      </c>
+      <c r="F10" s="0">
+        <v>18</v>
+      </c>
+      <c r="G10" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H10" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I10" s="0">
+        <v>18</v>
+      </c>
+      <c r="J10" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K10" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L10" s="0">
+        <v>1.0009898160494348</v>
+      </c>
+      <c r="M10" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="0">
+        <v>0.14999999999999999</v>
+      </c>
+      <c r="D11" s="0">
+        <v>0.25</v>
+      </c>
+      <c r="E11" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="F11" s="0">
+        <v>18</v>
+      </c>
+      <c r="G11" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H11" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I11" s="0">
+        <v>18</v>
+      </c>
+      <c r="J11" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K11" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L11" s="0">
+        <v>1.0004124233539311</v>
+      </c>
+      <c r="M11" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="0">
+        <v>0.45000000000000001</v>
+      </c>
+      <c r="D12" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="E12" s="0">
+        <v>0.25</v>
+      </c>
+      <c r="F12" s="0">
+        <v>18</v>
+      </c>
+      <c r="G12" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H12" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I12" s="0">
+        <v>18</v>
+      </c>
+      <c r="J12" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K12" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L12" s="0">
+        <v>1.0004949080247174</v>
+      </c>
+      <c r="M12" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="0">
+        <v>0.01</v>
+      </c>
+      <c r="D13" s="0">
+        <v>0.97999999999999998</v>
+      </c>
+      <c r="E13" s="0">
+        <v>0.01</v>
+      </c>
+      <c r="F13" s="0">
+        <v>18</v>
+      </c>
+      <c r="G13" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H13" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I13" s="0">
+        <v>19</v>
+      </c>
+      <c r="J13" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="K13" s="0">
+        <v>9.5666603908752492</v>
+      </c>
+      <c r="L13" s="0">
+        <v>1.0010632321660935</v>
+      </c>
+      <c r="M13" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" s="0"/>
+      <c r="D14" s="0"/>
+      <c r="E14" s="0"/>
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0">
+        <v>19</v>
+      </c>
+      <c r="J14" s="0">
+        <v>60.075372664158422</v>
+      </c>
+      <c r="K14" s="0">
+        <v>9.3953099878358124</v>
+      </c>
+      <c r="L14" s="0"/>
+      <c r="M14" s="0" t="s">
+        <v>134</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.125" customWidth="true"/>
+    <col min="2" max="2" width="67.125" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(q1): complete latest gravity-aligned artifacts and evidence
</commit_message>
<xml_diff>
--- a/results/q1_exact_dp/Q1_结果提交.xlsx
+++ b/results/q1_exact_dp/Q1_结果提交.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Q3_中继架次" sheetId="4" r:id="rId4"/>
     <sheet name="Q3_通信保障" sheetId="5" r:id="rId5"/>
     <sheet name="Q4_分区配置" sheetId="6" r:id="rId6"/>
+    <sheet name="Q1_方案对比" sheetId="7" r:id="rId10"/>
+    <sheet name="Q1_模型说明" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="151">
   <si>
     <r>
       <rPr>
@@ -664,6 +666,150 @@
   </si>
   <si>
     <t>S015-MED-01;S015-FOD-01;S015-WAT-01</t>
+  </si>
+  <si>
+    <t>objective</t>
+  </si>
+  <si>
+    <t>N-E-T</t>
+  </si>
+  <si>
+    <t>N-T-E</t>
+  </si>
+  <si>
+    <t>E-N-T</t>
+  </si>
+  <si>
+    <t>E-T-N</t>
+  </si>
+  <si>
+    <t>T-N-E</t>
+  </si>
+  <si>
+    <t>T-E-N</t>
+  </si>
+  <si>
+    <t>weighted_joint_N60_E25_T15</t>
+  </si>
+  <si>
+    <t>weighted_joint_balanced</t>
+  </si>
+  <si>
+    <t>weighted_joint_N15_E60_T25</t>
+  </si>
+  <si>
+    <t>weighted_joint_N15_E25_T60</t>
+  </si>
+  <si>
+    <t>weighted_joint_N45_E30_T25</t>
+  </si>
+  <si>
+    <t>weighted_joint_energy_dominant_N01_E98_T01</t>
+  </si>
+  <si>
+    <t>greedy_baseline</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>lexicographic</t>
+  </si>
+  <si>
+    <t>joint_weighted</t>
+  </si>
+  <si>
+    <t>greedy</t>
+  </si>
+  <si>
+    <t>sortie_weight</t>
+  </si>
+  <si>
+    <t>energy_weight</t>
+  </si>
+  <si>
+    <t>time_weight</t>
+  </si>
+  <si>
+    <t>scale_sorties</t>
+  </si>
+  <si>
+    <t>scale_energy_kWh</t>
+  </si>
+  <si>
+    <t>scale_time_h</t>
+  </si>
+  <si>
+    <t>total_sorties</t>
+  </si>
+  <si>
+    <t>total_energy_kWh</t>
+  </si>
+  <si>
+    <t>total_operation_time_h</t>
+  </si>
+  <si>
+    <t>normalized_objective</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>single-objective priority order</t>
+  </si>
+  <si>
+    <t>all three criteria included</t>
+  </si>
+  <si>
+    <t>baseline only</t>
+  </si>
+  <si>
+    <t>项目</t>
+  </si>
+  <si>
+    <t>重力加速度</t>
+  </si>
+  <si>
+    <t>算法</t>
+  </si>
+  <si>
+    <t>主方案</t>
+  </si>
+  <si>
+    <t>三目标加权</t>
+  </si>
+  <si>
+    <t>主方案结果</t>
+  </si>
+  <si>
+    <t>时间口径</t>
+  </si>
+  <si>
+    <t>最优性范围</t>
+  </si>
+  <si>
+    <t>说明</t>
+  </si>
+  <si>
+    <t>g=9.806 m/s^2，与问题二三统一</t>
+  </si>
+  <si>
+    <t>可行模式枚举 + 精确计数状态动态规划；intlinprog交叉验证</t>
+  </si>
+  <si>
+    <t>词典序：架次数 → 能耗 → 累计作业时间</t>
+  </si>
+  <si>
+    <t>J=wN*N/N0+wE*E/E0+wT*T/T0，权重和为1</t>
+  </si>
+  <si>
+    <t>18架次，59.130253926649 kWh，9.104448819143 h</t>
+  </si>
+  <si>
+    <t>模板往返时间列沿用完整架次作业时间；CSV另保留flight_time_s纯飞行时间</t>
+  </si>
+  <si>
+    <t>固定物理解释、枚举模式及数值容差下的所选目标；不代表所有偏好唯一最优</t>
   </si>
 </sst>
 </file>
@@ -1868,10 +2014,10 @@
         <v>1692.1690773290522</v>
       </c>
       <c r="H2" s="7">
-        <v>2.9175823075810157</v>
+        <v>2.9175399733426497</v>
       </c>
       <c r="I2" s="7">
-        <v>63.5302211552373</v>
+        <v>63.530750333216879</v>
       </c>
     </row>
     <row r="3">
@@ -1897,10 +2043,10 @@
         <v>1494.1690773290522</v>
       </c>
       <c r="H3" s="7">
-        <v>2.9957692627220123</v>
+        <v>2.9957264798521339</v>
       </c>
       <c r="I3" s="7">
-        <v>62.552884215974849</v>
+        <v>62.553419001848319</v>
       </c>
     </row>
     <row r="4">
@@ -1926,10 +2072,10 @@
         <v>1816.6943000984102</v>
       </c>
       <c r="H4" s="6">
-        <v>2.7134222874377589</v>
+        <v>2.7133881402010411</v>
       </c>
       <c r="I4" s="6">
-        <v>32.164442814056024</v>
+        <v>32.165296494973973</v>
       </c>
     </row>
     <row r="5">
@@ -1955,10 +2101,10 @@
         <v>2041.812384815207</v>
       </c>
       <c r="H5" s="6">
-        <v>5.7212246708574126</v>
+        <v>5.7211798054824712</v>
       </c>
       <c r="I5" s="6">
-        <v>28.484691614282344</v>
+        <v>28.48525243146911</v>
       </c>
     </row>
     <row r="6">
@@ -1984,10 +2130,10 @@
         <v>2080.5233035436581</v>
       </c>
       <c r="H6" s="6">
-        <v>2.7799174679726693</v>
+        <v>2.7798347763964069</v>
       </c>
       <c r="I6" s="6">
-        <v>30.502063300683268</v>
+        <v>30.504130590089829</v>
       </c>
     </row>
     <row r="7">
@@ -2013,10 +2159,10 @@
         <v>2370.0913496048561</v>
       </c>
       <c r="H7" s="6">
-        <v>5.7649651151972972</v>
+        <v>5.7648566851506047</v>
       </c>
       <c r="I7" s="6">
-        <v>27.937936060033785</v>
+        <v>27.939291435617442</v>
       </c>
     </row>
     <row r="8">
@@ -2042,10 +2188,10 @@
         <v>2301.0566924831601</v>
       </c>
       <c r="H8" s="6">
-        <v>6.1529320189069754</v>
+        <v>6.1528598719220176</v>
       </c>
       <c r="I8" s="6">
-        <v>23.088349763662809</v>
+        <v>23.08925160097478</v>
       </c>
     </row>
     <row r="9">
@@ -2071,10 +2217,10 @@
         <v>1877.1905245257485</v>
       </c>
       <c r="H9" s="6">
-        <v>4.2221928595068432</v>
+        <v>4.2221391566447011</v>
       </c>
       <c r="I9" s="6">
-        <v>47.222589256164461</v>
+        <v>47.223260541941237</v>
       </c>
     </row>
     <row r="10">
@@ -2100,10 +2246,10 @@
         <v>1561.553867961642</v>
       </c>
       <c r="H10" s="6">
-        <v>2.5979878649120525</v>
+        <v>2.5979349093557809</v>
       </c>
       <c r="I10" s="6">
-        <v>67.525151688599337</v>
+        <v>67.525813633052749</v>
       </c>
     </row>
     <row r="11">
@@ -2129,10 +2275,10 @@
         <v>1907.5664573299073</v>
       </c>
       <c r="H11" s="6">
-        <v>3.4108943800033673</v>
+        <v>3.4108086087645568</v>
       </c>
       <c r="I11" s="6">
-        <v>57.363820249957911</v>
+        <v>57.364892390443046</v>
       </c>
     </row>
     <row r="12">
@@ -2158,10 +2304,10 @@
         <v>2199.7012130854737</v>
       </c>
       <c r="H12" s="6">
-        <v>5.8360117114838781</v>
+        <v>5.8359572284520809</v>
       </c>
       <c r="I12" s="6">
-        <v>27.049853606451524</v>
+        <v>27.050534644348989</v>
       </c>
     </row>
     <row r="13">
@@ -2187,10 +2333,10 @@
         <v>1558.4417330887577</v>
       </c>
       <c r="H13" s="6">
-        <v>2.096233734426161</v>
+        <v>2.0962044018931136</v>
       </c>
       <c r="I13" s="6">
-        <v>47.594156639345975</v>
+        <v>47.594889952672162</v>
       </c>
     </row>
     <row r="14">
@@ -2216,10 +2362,10 @@
         <v>1555.3795658312195</v>
       </c>
       <c r="H14" s="6">
-        <v>1.8231956980899264</v>
+        <v>1.8231444995358754</v>
       </c>
       <c r="I14" s="6">
-        <v>54.42010754775184</v>
+        <v>54.421387511603115</v>
       </c>
     </row>
     <row r="15">
@@ -2245,10 +2391,10 @@
         <v>1188.4204722350105</v>
       </c>
       <c r="H15" s="6">
-        <v>1.0739517654350652</v>
+        <v>1.0739201272065426</v>
       </c>
       <c r="I15" s="6">
-        <v>73.151205864123369</v>
+        <v>73.151996819836441</v>
       </c>
     </row>
     <row r="16">
@@ -2274,10 +2420,10 @@
         <v>1922.7403507441504</v>
       </c>
       <c r="H16" s="6">
-        <v>2.7524142988016456</v>
+        <v>2.752361240693304</v>
       </c>
       <c r="I16" s="6">
-        <v>31.18964252995886</v>
+        <v>31.1909689826674</v>
       </c>
     </row>
     <row r="17">
@@ -2303,10 +2449,10 @@
         <v>1510.4723251019025</v>
       </c>
       <c r="H17" s="6">
-        <v>1.8247592723274209</v>
+        <v>1.8247168036813126</v>
       </c>
       <c r="I17" s="6">
-        <v>54.381018191814476</v>
+        <v>54.382079907967181</v>
       </c>
     </row>
     <row r="18">
@@ -2332,10 +2478,10 @@
         <v>1869.7564163814459</v>
       </c>
       <c r="H18" s="6">
-        <v>2.1403884821071424</v>
+        <v>2.1402998341980486</v>
       </c>
       <c r="I18" s="6">
-        <v>46.490287947321441</v>
+        <v>46.492504145048784</v>
       </c>
     </row>
     <row r="19">
@@ -2361,10 +2507,10 @@
         <v>1828.2766374270207</v>
       </c>
       <c r="H19" s="6">
-        <v>2.3074528242842076</v>
+        <v>2.3073813838759016</v>
       </c>
       <c r="I19" s="6">
-        <v>42.313679392894812</v>
+        <v>42.315465403102458</v>
       </c>
     </row>
   </sheetData>
@@ -6080,4 +6226,581 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="41.82421875" customWidth="true"/>
+    <col min="2" max="2" width="13.22265625" customWidth="true"/>
+    <col min="3" max="3" width="12.625" customWidth="true"/>
+    <col min="4" max="4" width="13.5234375" customWidth="true"/>
+    <col min="5" max="5" width="12.625" customWidth="true"/>
+    <col min="6" max="6" width="11.921875" customWidth="true"/>
+    <col min="7" max="7" width="17.22265625" customWidth="true"/>
+    <col min="8" max="8" width="12.125" customWidth="true"/>
+    <col min="9" max="9" width="10.82421875" customWidth="true"/>
+    <col min="10" max="10" width="16.125" customWidth="true"/>
+    <col min="11" max="11" width="19.921875" customWidth="true"/>
+    <col min="12" max="12" width="18.921875" customWidth="true"/>
+    <col min="13" max="13" width="25.22265625" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+      <c r="I2" s="0">
+        <v>18</v>
+      </c>
+      <c r="J2" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K2" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L2" s="0"/>
+      <c r="M2" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0">
+        <v>18</v>
+      </c>
+      <c r="J3" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K3" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L3" s="0"/>
+      <c r="M3" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0">
+        <v>19</v>
+      </c>
+      <c r="J4" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="K4" s="0">
+        <v>9.5666603908752492</v>
+      </c>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="0"/>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+      <c r="I5" s="0">
+        <v>19</v>
+      </c>
+      <c r="J5" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="K5" s="0">
+        <v>9.5666603908752492</v>
+      </c>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+      <c r="I6" s="0">
+        <v>18</v>
+      </c>
+      <c r="J6" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K6" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L6" s="0"/>
+      <c r="M6" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="0"/>
+      <c r="D7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0">
+        <v>18</v>
+      </c>
+      <c r="J7" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K7" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0.25</v>
+      </c>
+      <c r="E8" s="0">
+        <v>0.14999999999999999</v>
+      </c>
+      <c r="F8" s="0">
+        <v>18</v>
+      </c>
+      <c r="G8" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H8" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I8" s="0">
+        <v>18</v>
+      </c>
+      <c r="J8" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K8" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L8" s="0">
+        <v>1.0004124233539311</v>
+      </c>
+      <c r="M8" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="0">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D9" s="0">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E9" s="0">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F9" s="0">
+        <v>18</v>
+      </c>
+      <c r="G9" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H9" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I9" s="0">
+        <v>18</v>
+      </c>
+      <c r="J9" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K9" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L9" s="0">
+        <v>1.0005498978052414</v>
+      </c>
+      <c r="M9" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="0">
+        <v>0.14999999999999999</v>
+      </c>
+      <c r="D10" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="E10" s="0">
+        <v>0.25</v>
+      </c>
+      <c r="F10" s="0">
+        <v>18</v>
+      </c>
+      <c r="G10" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H10" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I10" s="0">
+        <v>18</v>
+      </c>
+      <c r="J10" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K10" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L10" s="0">
+        <v>1.0009898160494348</v>
+      </c>
+      <c r="M10" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="0">
+        <v>0.14999999999999999</v>
+      </c>
+      <c r="D11" s="0">
+        <v>0.25</v>
+      </c>
+      <c r="E11" s="0">
+        <v>0.59999999999999998</v>
+      </c>
+      <c r="F11" s="0">
+        <v>18</v>
+      </c>
+      <c r="G11" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H11" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I11" s="0">
+        <v>18</v>
+      </c>
+      <c r="J11" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K11" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L11" s="0">
+        <v>1.0004124233539311</v>
+      </c>
+      <c r="M11" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="0">
+        <v>0.45000000000000001</v>
+      </c>
+      <c r="D12" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="E12" s="0">
+        <v>0.25</v>
+      </c>
+      <c r="F12" s="0">
+        <v>18</v>
+      </c>
+      <c r="G12" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H12" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I12" s="0">
+        <v>18</v>
+      </c>
+      <c r="J12" s="0">
+        <v>59.130253926648535</v>
+      </c>
+      <c r="K12" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="L12" s="0">
+        <v>1.0004949080247174</v>
+      </c>
+      <c r="M12" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="0">
+        <v>0.01</v>
+      </c>
+      <c r="D13" s="0">
+        <v>0.97999999999999998</v>
+      </c>
+      <c r="E13" s="0">
+        <v>0.01</v>
+      </c>
+      <c r="F13" s="0">
+        <v>18</v>
+      </c>
+      <c r="G13" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="H13" s="0">
+        <v>9.1044488191432436</v>
+      </c>
+      <c r="I13" s="0">
+        <v>19</v>
+      </c>
+      <c r="J13" s="0">
+        <v>59.032867793338525</v>
+      </c>
+      <c r="K13" s="0">
+        <v>9.5666603908752492</v>
+      </c>
+      <c r="L13" s="0">
+        <v>1.0010632321660935</v>
+      </c>
+      <c r="M13" s="0" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" s="0"/>
+      <c r="D14" s="0"/>
+      <c r="E14" s="0"/>
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0">
+        <v>19</v>
+      </c>
+      <c r="J14" s="0">
+        <v>60.075372664158422</v>
+      </c>
+      <c r="K14" s="0">
+        <v>9.3953099878358124</v>
+      </c>
+      <c r="L14" s="0"/>
+      <c r="M14" s="0" t="s">
+        <v>134</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.125" customWidth="true"/>
+    <col min="2" max="2" width="67.125" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>